<commit_message>
Add evaluation reports and update question retrieval for Django REST framework and Playwright
- Introduced new evaluation report files for Django REST framework and Playwright in Excel format.
- Updated `generate_evaluation_report.py` to change the data directory to `django-rest-framework`.
- Enhanced JSON files for question retrieval with detailed LLM responses and cost metrics.
- Added new question datasets for LLM retrieval in the `llm_evaluation` directory, improving data evaluation capabilities.
</commit_message>
<xml_diff>
--- a/data_evaluation/playwright/evaluation_report_playwright.xlsx
+++ b/data_evaluation/playwright/evaluation_report_playwright.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sagundevkota/Documents/opensource/hierarchical-rag/data_evaluation/playwright/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A405149-57E4-9B4B-AC3C-47940FB4B5A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E635B22F-2D34-BF4E-9BD1-38AB6C5CEA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="34">
   <si>
     <t>question_type</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>rouge_score(mode=recall)</t>
+  </si>
+  <si>
+    <t>context_length</t>
   </si>
   <si>
     <t>llm_calls</t>
@@ -134,9 +137,6 @@
   <si>
     <t>Total Tokens (per query) (lower is better)</t>
   </si>
-  <si>
-    <t>Generation Tokens (per query) (lower is better)</t>
-  </si>
 </sst>
 </file>
 
@@ -164,7 +164,7 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -172,7 +172,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -199,7 +199,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -210,8 +210,17 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color auto="1"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -220,41 +229,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -309,7 +305,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Context Precision</a:t>
+              <a:t>Context Precision by Question Type (higher is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -401,23 +397,23 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.63290000000000002</c:v>
+                  <c:v>0.90469999999999995</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.68640000000000001</c:v>
+                  <c:v>0.83199999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.81699999999999995</c:v>
+                  <c:v>0.96060000000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.76580000000000004</c:v>
+                  <c:v>0.86199999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DA69-8D4F-BD15-12EE9BA8EB43}"/>
+              <c16:uniqueId val="{00000000-F6BD-8B42-B37F-FA7DFFF57367}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -488,7 +484,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-DA69-8D4F-BD15-12EE9BA8EB43}"/>
+              <c16:uniqueId val="{00000001-F6BD-8B42-B37F-FA7DFFF57367}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -559,7 +555,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-DA69-8D4F-BD15-12EE9BA8EB43}"/>
+              <c16:uniqueId val="{00000002-F6BD-8B42-B37F-FA7DFFF57367}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -573,11 +569,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1781725135"/>
-        <c:axId val="1781726847"/>
+        <c:axId val="2017532656"/>
+        <c:axId val="2017476736"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1781725135"/>
+        <c:axId val="2017532656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -620,7 +616,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1781726847"/>
+        <c:crossAx val="2017476736"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -628,7 +624,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1781726847"/>
+        <c:axId val="2017476736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -679,7 +675,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1781725135"/>
+        <c:crossAx val="2017532656"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -801,7 +797,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Context Recall</a:t>
+              <a:t>Context Recall by Question Type (higher is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -893,23 +889,23 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.84</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.87729999999999997</c:v>
+                  <c:v>0.93030000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.94799999999999995</c:v>
+                  <c:v>0.97199999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.87</c:v>
+                  <c:v>0.98</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A616-7341-BBA5-ED23AE112421}"/>
+              <c16:uniqueId val="{00000000-5191-EE49-8E7E-A1A0D4BFF44A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -980,7 +976,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A616-7341-BBA5-ED23AE112421}"/>
+              <c16:uniqueId val="{00000001-5191-EE49-8E7E-A1A0D4BFF44A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1051,7 +1047,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-A616-7341-BBA5-ED23AE112421}"/>
+              <c16:uniqueId val="{00000002-5191-EE49-8E7E-A1A0D4BFF44A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1065,11 +1061,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="343475631"/>
-        <c:axId val="343464831"/>
+        <c:axId val="1969310784"/>
+        <c:axId val="1969312496"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="343475631"/>
+        <c:axId val="1969310784"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1112,7 +1108,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="343464831"/>
+        <c:crossAx val="1969312496"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1120,7 +1116,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="343464831"/>
+        <c:axId val="1969312496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1171,7 +1167,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="343475631"/>
+        <c:crossAx val="1969310784"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1293,7 +1289,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Answer Accuracy</a:t>
+              <a:t>Answer Accuracy by Question Type (higher is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1385,23 +1381,23 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.72</c:v>
+                  <c:v>0.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0.94</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.96</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.84</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5045-2B41-82C6-951CF6738547}"/>
+              <c16:uniqueId val="{00000000-2BB5-2D47-8A79-79EFD5AB30D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1472,7 +1468,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-5045-2B41-82C6-951CF6738547}"/>
+              <c16:uniqueId val="{00000001-2BB5-2D47-8A79-79EFD5AB30D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1543,7 +1539,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-5045-2B41-82C6-951CF6738547}"/>
+              <c16:uniqueId val="{00000002-2BB5-2D47-8A79-79EFD5AB30D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1557,11 +1553,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1827447759"/>
-        <c:axId val="1827449471"/>
+        <c:axId val="1926472368"/>
+        <c:axId val="1926474080"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1827447759"/>
+        <c:axId val="1926472368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1604,7 +1600,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1827449471"/>
+        <c:crossAx val="1926474080"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1612,7 +1608,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1827449471"/>
+        <c:axId val="1926474080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1663,7 +1659,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1827447759"/>
+        <c:crossAx val="1926472368"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1785,7 +1781,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Helpfulness</a:t>
+              <a:t>Helpfulness by Question Type (higher is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1877,23 +1873,23 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4.4400000000000004</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.92</c:v>
+                  <c:v>4.88</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.8</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3F49-CE42-92A1-8A1035668C21}"/>
+              <c16:uniqueId val="{00000000-13D6-864F-814A-011C3D84AD04}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1964,7 +1960,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3F49-CE42-92A1-8A1035668C21}"/>
+              <c16:uniqueId val="{00000001-13D6-864F-814A-011C3D84AD04}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2035,7 +2031,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3F49-CE42-92A1-8A1035668C21}"/>
+              <c16:uniqueId val="{00000002-13D6-864F-814A-011C3D84AD04}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2049,11 +2045,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1826987951"/>
-        <c:axId val="1826989663"/>
+        <c:axId val="374460800"/>
+        <c:axId val="374462512"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1826987951"/>
+        <c:axId val="374460800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2096,7 +2092,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826989663"/>
+        <c:crossAx val="374462512"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2104,7 +2100,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1826989663"/>
+        <c:axId val="374462512"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2155,7 +2151,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826987951"/>
+        <c:crossAx val="374460800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2277,7 +2273,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Factual Correctness</a:t>
+              <a:t>Factual Correctness by Question Type (higher is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2369,23 +2365,23 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.44</c:v>
+                  <c:v>0.52959999999999996</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.55600000000000005</c:v>
+                  <c:v>0.52959999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.56000000000000005</c:v>
+                  <c:v>0.48880000000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.58919999999999995</c:v>
+                  <c:v>0.65959999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F11F-0946-88CE-EDF6EB280EF3}"/>
+              <c16:uniqueId val="{00000000-6CA7-334B-AA44-EEFA8C047D0F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2456,7 +2452,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-F11F-0946-88CE-EDF6EB280EF3}"/>
+              <c16:uniqueId val="{00000001-6CA7-334B-AA44-EEFA8C047D0F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2527,7 +2523,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-F11F-0946-88CE-EDF6EB280EF3}"/>
+              <c16:uniqueId val="{00000002-6CA7-334B-AA44-EEFA8C047D0F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2541,11 +2537,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1826896399"/>
-        <c:axId val="1826898111"/>
+        <c:axId val="376261600"/>
+        <c:axId val="376227792"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1826896399"/>
+        <c:axId val="376261600"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2588,7 +2584,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826898111"/>
+        <c:crossAx val="376227792"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2596,7 +2592,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1826898111"/>
+        <c:axId val="376227792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2647,7 +2643,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826896399"/>
+        <c:crossAx val="376261600"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2769,7 +2765,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Total Cost</a:t>
+              <a:t>Total Cost by Question Type (lower is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2861,23 +2857,23 @@
                 <c:formatCode>[$$-409]0.000000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>7.9469999999999992E-3</c:v>
+                  <c:v>8.9099999999999997E-4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.3489999999999997E-3</c:v>
+                  <c:v>1.33E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.6020000000000003E-3</c:v>
+                  <c:v>1.32E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.9840000000000007E-3</c:v>
+                  <c:v>1.0510000000000001E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A289-7F4C-997F-46B4DEF13845}"/>
+              <c16:uniqueId val="{00000000-C005-9649-B606-0E12ABCA9C3B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2948,7 +2944,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A289-7F4C-997F-46B4DEF13845}"/>
+              <c16:uniqueId val="{00000001-C005-9649-B606-0E12ABCA9C3B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3019,7 +3015,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-A289-7F4C-997F-46B4DEF13845}"/>
+              <c16:uniqueId val="{00000002-C005-9649-B606-0E12ABCA9C3B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3033,11 +3029,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1826679951"/>
-        <c:axId val="1826669615"/>
+        <c:axId val="563171872"/>
+        <c:axId val="563173584"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1826679951"/>
+        <c:axId val="563171872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3080,7 +3076,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826669615"/>
+        <c:crossAx val="563173584"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3088,7 +3084,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1826669615"/>
+        <c:axId val="563173584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3139,7 +3135,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1826679951"/>
+        <c:crossAx val="563171872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3261,7 +3257,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Generation Cost</a:t>
+              <a:t>Generation Cost by Question Type (lower is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3353,23 +3349,23 @@
                 <c:formatCode>[$$-409]0.000000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>5.2700000000000002E-4</c:v>
+                  <c:v>8.9099999999999997E-4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.9400000000000009E-4</c:v>
+                  <c:v>1.33E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.8599999999999996E-4</c:v>
+                  <c:v>1.32E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.8400000000000004E-4</c:v>
+                  <c:v>1.0510000000000001E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-15EE-3A4C-971D-71239B159084}"/>
+              <c16:uniqueId val="{00000000-5ED8-3A45-A768-E655C2E60892}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3440,7 +3436,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-15EE-3A4C-971D-71239B159084}"/>
+              <c16:uniqueId val="{00000001-5ED8-3A45-A768-E655C2E60892}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3511,7 +3507,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-15EE-3A4C-971D-71239B159084}"/>
+              <c16:uniqueId val="{00000002-5ED8-3A45-A768-E655C2E60892}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3525,11 +3521,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="754701119"/>
-        <c:axId val="754499871"/>
+        <c:axId val="1079981024"/>
+        <c:axId val="1923483792"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="754701119"/>
+        <c:axId val="1079981024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3572,7 +3568,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="754499871"/>
+        <c:crossAx val="1923483792"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3580,7 +3576,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="754499871"/>
+        <c:axId val="1923483792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3631,7 +3627,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="754701119"/>
+        <c:crossAx val="1079981024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3753,7 +3749,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Total Tokens</a:t>
+              <a:t>Total Tokens by Question Type (lower is better)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3845,23 +3841,23 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>30420.48</c:v>
+                  <c:v>41182.92</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>35315.279999999999</c:v>
+                  <c:v>40293.08</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>32730.76</c:v>
+                  <c:v>40745.599999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>34701.68</c:v>
+                  <c:v>44095.88</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0CF3-874B-A1E1-4BB1FF35815B}"/>
+              <c16:uniqueId val="{00000000-1EEC-0143-820B-EC22B7CAF440}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3932,7 +3928,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0CF3-874B-A1E1-4BB1FF35815B}"/>
+              <c16:uniqueId val="{00000001-1EEC-0143-820B-EC22B7CAF440}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4003,7 +3999,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-0CF3-874B-A1E1-4BB1FF35815B}"/>
+              <c16:uniqueId val="{00000002-1EEC-0143-820B-EC22B7CAF440}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4017,11 +4013,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="754879391"/>
-        <c:axId val="754795631"/>
+        <c:axId val="563812672"/>
+        <c:axId val="563649952"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="754879391"/>
+        <c:axId val="563812672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4064,7 +4060,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="754795631"/>
+        <c:crossAx val="563649952"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4072,7 +4068,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="754795631"/>
+        <c:axId val="563649952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4123,499 +4119,7 @@
             <a:endParaRPr lang="en-NP"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="754879391"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-NP"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-NP"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Generation Tokens</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-NP"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$68</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>LLM Retriever</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$69:$A$72</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>straightforward</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>multi_hop</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>intent_driven</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>debugging</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$B$69:$B$72</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>1374.52</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2514.6799999999998</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2076.88</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1875.72</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6787-914B-A9B5-33BE7CD6DC56}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$68</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Naive RAG</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$69:$A$72</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>straightforward</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>multi_hop</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>intent_driven</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>debugging</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$C$69:$C$72</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>2243.88</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2297.3200000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2285.2800000000002</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2308.16</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6787-914B-A9B5-33BE7CD6DC56}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$D$68</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>RAPTOR</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$A$69:$A$72</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>straightforward</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>multi_hop</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>intent_driven</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>debugging</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$D$69:$D$72</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>2126.12</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2391.6799999999998</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2403.8000000000002</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2378</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6787-914B-A9B5-33BE7CD6DC56}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="754721375"/>
-        <c:axId val="754723087"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="754721375"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-NP"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="754723087"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="754723087"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-NP"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="754721375"/>
+        <c:crossAx val="563812672"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5022,46 +4526,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -8584,509 +8048,6 @@
 </file>
 
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -9595,21 +8556,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="2" name="Context Precision">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DA51C71-1A54-2A58-92C4-64A8D1CA2E75}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDD0AB94-F338-1D15-66D3-3B049240F88B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9631,21 +8592,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="3" name="Context Recall">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F631046E-DDAA-FA8D-4560-C1B5DE7B6CC5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5D03E02-CF64-ACAF-54B7-CABB9FC02198}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9667,21 +8628,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="4" name="Answer Accuracy">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B81A544D-49DF-F439-FA25-4CB3E8B08A98}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43A87E25-BA90-2D15-6A88-A686510A208E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9703,21 +8664,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
+        <xdr:cNvPr id="5" name="Helpfulness">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{924F2D13-50DD-0186-3AC5-DB1C6418B729}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C48BEF2B-EF68-776F-1D27-0A17EA56D8EC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9739,21 +8700,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>78</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5">
+        <xdr:cNvPr id="6" name="Factual Correctness">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B049B061-751C-C19C-A7B8-DCC0297DAC66}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF1768DE-95C1-A342-1F15-563D4850F6F1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9775,21 +8736,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>93</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Chart 6">
+        <xdr:cNvPr id="7" name="Total Cost">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00BF04E1-9AAD-8678-A329-7BB10A8AFB13}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1F0A888-71BF-00CC-DB1E-B4EB3A3F0DDC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9811,21 +8772,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>94</xdr:row>
+      <xdr:row>109</xdr:row>
       <xdr:rowOff>88900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>109</xdr:row>
+      <xdr:row>126</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="8" name="Chart 7">
+        <xdr:cNvPr id="8" name="Generation Cost">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F37EAAC1-1829-F837-A331-0162C6317A3C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1EC302AA-6B61-1BC9-88ED-D1670FB75318}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9847,21 +8808,21 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>109</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:row>127</xdr:row>
+      <xdr:rowOff>88900</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>124</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="9" name="Chart 8">
+        <xdr:cNvPr id="9" name="Total Tokens">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38F025EE-8CC7-84BD-1EFD-06F60E5208A2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{259BC723-577C-AEF5-15C4-323D746FEAB3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9874,42 +8835,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>125</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>139</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="10" name="Chart 9">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8C2870F-BC8C-FABC-5BE4-647D74A0287E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10210,13 +9135,13 @@
 </file>
 
 <file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{F6629CE7-843A-1949-98C8-8AB192AC6F7B}">
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{91CB7E68-7A9A-1B46-AE3A-CE07D30CF579}">
   <we:reference id="wa200010725" version="1.0.0.1" store="en-US" storeType="OMEX"/>
   <we:alternateReferences>
     <we:reference id="WA200010725" version="1.0.0.1" store="en-US" storeType="OMEX"/>
   </we:alternateReferences>
   <we:properties>
-    <we:property name="claude.fileId" value="&quot;17659aab-0990-436e-961c-e1881579552a&quot;"/>
+    <we:property name="claude.fileId" value="&quot;47dc475a-fd48-4b9e-9376-471366435d9f&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -10225,7 +9150,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -10237,16 +9162,17 @@
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10295,74 +9221,80 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.90469999999999995</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.86</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.52959999999999996</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.15279999999999999</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0.51100000000000001</v>
+      </c>
+      <c r="J2">
+        <v>6601.52</v>
+      </c>
+      <c r="K2">
+        <v>4.12</v>
+      </c>
+      <c r="L2">
+        <v>8.9099999999999997E-4</v>
+      </c>
+      <c r="M2">
+        <v>41182.92</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>38486.120000000003</v>
+      </c>
+      <c r="P2">
+        <v>8.9099999999999997E-4</v>
+      </c>
+      <c r="Q2">
+        <v>2696.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="1">
-        <v>0.63290000000000002</v>
-      </c>
-      <c r="D2">
-        <v>0.84</v>
-      </c>
-      <c r="E2">
-        <v>4.4400000000000004</v>
-      </c>
-      <c r="F2">
-        <v>0.72</v>
-      </c>
-      <c r="G2">
-        <v>0.44</v>
-      </c>
-      <c r="H2" s="1">
-        <v>0.14699999999999999</v>
-      </c>
-      <c r="I2">
-        <v>0.41549999999999998</v>
-      </c>
-      <c r="J2">
-        <v>3.56</v>
-      </c>
-      <c r="K2">
-        <v>7.9469999999999992E-3</v>
-      </c>
-      <c r="L2">
-        <v>30420.48</v>
-      </c>
-      <c r="M2">
-        <v>7.4209999999999996E-3</v>
-      </c>
-      <c r="N2">
-        <v>29045.96</v>
-      </c>
-      <c r="O2" s="1">
-        <v>5.2700000000000002E-4</v>
-      </c>
-      <c r="P2" s="1">
-        <v>1374.52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3">
         <v>0.60140000000000005</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>0.88</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>4.6399999999999997</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>0.8</v>
       </c>
       <c r="G3">
@@ -10371,31 +9303,34 @@
       <c r="H3">
         <v>0.13070000000000001</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3">
         <v>0.44400000000000001</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="1">
+        <v>5760.08</v>
+      </c>
+      <c r="K3">
         <v>1</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>7.4700000000000005E-4</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>2243.88</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>7.4700000000000005E-4</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>2243.88</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>0.61529999999999996</v>
@@ -10409,7 +9344,7 @@
       <c r="F4">
         <v>0.81</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>0.52759999999999996</v>
       </c>
       <c r="H4">
@@ -10419,77 +9354,83 @@
         <v>0.43890000000000001</v>
       </c>
       <c r="J4">
+        <v>5976.8</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
-      <c r="K4" s="1">
+      <c r="L4" s="1">
         <v>6.9700000000000003E-4</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
         <v>2126.12</v>
       </c>
-      <c r="O4">
+      <c r="P4" s="1">
         <v>6.9700000000000003E-4</v>
       </c>
-      <c r="P4">
+      <c r="Q4" s="1">
         <v>2126.12</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="1">
-        <v>0.68640000000000001</v>
+        <v>0.83199999999999996</v>
       </c>
       <c r="D5" s="1">
-        <v>0.87729999999999997</v>
+        <v>0.93030000000000002</v>
       </c>
       <c r="E5">
-        <v>4.92</v>
+        <v>4.88</v>
       </c>
       <c r="F5" s="1">
-        <v>0.94</v>
+        <v>0.95</v>
       </c>
       <c r="G5" s="1">
-        <v>0.55600000000000005</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0.15629999999999999</v>
+        <v>0.52959999999999996</v>
+      </c>
+      <c r="H5">
+        <v>0.13800000000000001</v>
       </c>
       <c r="I5" s="1">
-        <v>0.37440000000000001</v>
+        <v>0.38879999999999998</v>
       </c>
       <c r="J5">
-        <v>3.92</v>
+        <v>9502.1200000000008</v>
       </c>
       <c r="K5">
-        <v>9.3489999999999997E-3</v>
-      </c>
-      <c r="L5">
-        <v>35315.279999999999</v>
+        <v>3.96</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1.33E-3</v>
       </c>
       <c r="M5">
-        <v>8.3549999999999996E-3</v>
+        <v>40293.08</v>
       </c>
       <c r="N5">
-        <v>32800.6</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>9.9400000000000009E-4</v>
-      </c>
-      <c r="P5">
-        <v>2514.6799999999998</v>
+        <v>36678.32</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1.33E-3</v>
+      </c>
+      <c r="Q5">
+        <v>3614.76</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>0.50339999999999996</v>
@@ -10506,34 +9447,37 @@
       <c r="G6">
         <v>0.41639999999999999</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <v>0.1542</v>
       </c>
       <c r="I6">
         <v>0.33389999999999997</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="1">
+        <v>5731.36</v>
+      </c>
+      <c r="K6">
         <v>1</v>
       </c>
-      <c r="K6" s="1">
+      <c r="L6">
         <v>8.8500000000000004E-4</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="1">
         <v>2297.3200000000002</v>
       </c>
-      <c r="O6" s="1">
+      <c r="P6">
         <v>8.8500000000000004E-4</v>
       </c>
-      <c r="P6" s="1">
+      <c r="Q6" s="1">
         <v>2297.3200000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
       </c>
       <c r="C7">
         <v>0.58909999999999996</v>
@@ -10557,77 +9501,83 @@
         <v>0.32250000000000001</v>
       </c>
       <c r="J7">
+        <v>6316.64</v>
+      </c>
+      <c r="K7">
         <v>1</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>8.9800000000000004E-4</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>2391.6799999999998</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>8.9800000000000004E-4</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>2391.6799999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1">
-        <v>0.81699999999999995</v>
+        <v>0.96060000000000001</v>
       </c>
       <c r="D8" s="1">
-        <v>0.94799999999999995</v>
+        <v>0.97199999999999998</v>
       </c>
       <c r="E8" s="1">
         <v>5</v>
       </c>
       <c r="F8" s="1">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="G8" s="1">
-        <v>0.56000000000000005</v>
+        <v>0.48880000000000001</v>
       </c>
       <c r="H8">
-        <v>0.14549999999999999</v>
+        <v>0.1225</v>
       </c>
       <c r="I8" s="1">
-        <v>0.45829999999999999</v>
+        <v>0.47939999999999999</v>
       </c>
       <c r="J8">
-        <v>3.52</v>
+        <v>8889.7999999999993</v>
       </c>
       <c r="K8">
-        <v>8.6020000000000003E-3</v>
-      </c>
-      <c r="L8">
-        <v>32730.76</v>
+        <v>4.12</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1.32E-3</v>
       </c>
       <c r="M8">
-        <v>7.7159999999999998E-3</v>
+        <v>40745.599999999999</v>
       </c>
       <c r="N8">
-        <v>30653.88</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>8.8599999999999996E-4</v>
+        <v>37246.04</v>
       </c>
       <c r="P8" s="1">
-        <v>2076.88</v>
+        <v>1.32E-3</v>
+      </c>
+      <c r="Q8">
+        <v>3499.56</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9">
         <v>0.59199999999999997</v>
@@ -10650,28 +9600,31 @@
       <c r="I9">
         <v>0.40189999999999998</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="1">
+        <v>5638.32</v>
+      </c>
+      <c r="K9">
         <v>1</v>
       </c>
-      <c r="K9" s="1">
+      <c r="L9">
         <v>8.2299999999999995E-4</v>
       </c>
-      <c r="L9" s="1">
+      <c r="M9" s="1">
         <v>2285.2800000000002</v>
       </c>
-      <c r="O9" s="1">
+      <c r="P9">
         <v>8.2299999999999995E-4</v>
       </c>
-      <c r="P9">
+      <c r="Q9" s="1">
         <v>2285.2800000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10">
         <v>0.66749999999999998</v>
@@ -10695,85 +9648,91 @@
         <v>0.40799999999999997</v>
       </c>
       <c r="J10">
+        <v>6178.72</v>
+      </c>
+      <c r="K10">
         <v>1</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>8.7200000000000005E-4</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>2403.8000000000002</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>8.7200000000000005E-4</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>2403.8000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" s="1">
-        <v>0.76580000000000004</v>
-      </c>
-      <c r="D11">
-        <v>0.87</v>
-      </c>
-      <c r="E11">
-        <v>4.8</v>
-      </c>
-      <c r="F11">
-        <v>0.84</v>
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="E11" s="1">
+        <v>5</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.94</v>
       </c>
       <c r="G11">
-        <v>0.58919999999999995</v>
+        <v>0.65959999999999996</v>
       </c>
       <c r="H11">
-        <v>0.16689999999999999</v>
-      </c>
-      <c r="I11">
-        <v>0.4052</v>
+        <v>0.16420000000000001</v>
+      </c>
+      <c r="I11" s="1">
+        <v>0.45779999999999998</v>
       </c>
       <c r="J11">
-        <v>3.72</v>
+        <v>8029.8</v>
       </c>
       <c r="K11">
-        <v>8.9840000000000007E-3</v>
+        <v>3.88</v>
       </c>
       <c r="L11">
-        <v>34701.68</v>
+        <v>1.0510000000000001E-3</v>
       </c>
       <c r="M11">
-        <v>8.3000000000000001E-3</v>
+        <v>44095.88</v>
       </c>
       <c r="N11">
-        <v>32825.96</v>
-      </c>
-      <c r="O11" s="1">
-        <v>6.8400000000000004E-4</v>
-      </c>
-      <c r="P11" s="1">
-        <v>1875.72</v>
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>40902.199999999997</v>
+      </c>
+      <c r="P11">
+        <v>1.0510000000000001E-3</v>
+      </c>
+      <c r="Q11">
+        <v>3193.68</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>0.71950000000000003</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>0.96330000000000005</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12">
         <v>4.92</v>
       </c>
       <c r="F12" s="1">
@@ -10788,28 +9747,31 @@
       <c r="I12">
         <v>0.4088</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="1">
+        <v>5730.24</v>
+      </c>
+      <c r="K12">
         <v>1</v>
       </c>
-      <c r="K12" s="1">
+      <c r="L12" s="1">
         <v>7.5600000000000005E-4</v>
       </c>
-      <c r="L12" s="1">
+      <c r="M12" s="1">
         <v>2308.16</v>
       </c>
-      <c r="O12">
+      <c r="P12" s="1">
         <v>7.5600000000000005E-4</v>
       </c>
-      <c r="P12">
+      <c r="Q12" s="1">
         <v>2308.16</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13">
         <v>0.73319999999999996</v>
@@ -10829,22 +9791,25 @@
       <c r="H13" s="1">
         <v>0.1946</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>0.42609999999999998</v>
       </c>
       <c r="J13">
+        <v>5997.4</v>
+      </c>
+      <c r="K13">
         <v>1</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>7.9100000000000004E-4</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>2378</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>7.9100000000000004E-4</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>2378</v>
       </c>
     </row>
@@ -10854,41 +9819,46 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C874811-0192-7049-A49E-14BD1B5B973D}">
-  <dimension ref="A1:D72"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50A7A716-9B22-C14C-8654-C6FDBAD1D418}">
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="40.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>25</v>
+      <c r="A4" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>16</v>
+      <c r="A5" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="B5" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A5,'RAG Comparison'!$B$2:$B$13,B$4)</f>
-        <v>0.63290000000000002</v>
+        <v>0.90469999999999995</v>
       </c>
       <c r="C5" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A5,'RAG Comparison'!$B$2:$B$13,C$4)</f>
@@ -10901,81 +9871,81 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="6">
+        <v>21</v>
+      </c>
+      <c r="B6" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A6,'RAG Comparison'!$B$2:$B$13,B$4)</f>
-        <v>0.68640000000000001</v>
-      </c>
-      <c r="C6" s="6">
+        <v>0.83199999999999996</v>
+      </c>
+      <c r="C6" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A6,'RAG Comparison'!$B$2:$B$13,C$4)</f>
         <v>0.50339999999999996</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A6,'RAG Comparison'!$B$2:$B$13,D$4)</f>
         <v>0.58909999999999996</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="6">
+        <v>22</v>
+      </c>
+      <c r="B7" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A7,'RAG Comparison'!$B$2:$B$13,B$4)</f>
-        <v>0.81699999999999995</v>
-      </c>
-      <c r="C7" s="6">
+        <v>0.96060000000000001</v>
+      </c>
+      <c r="C7" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A7,'RAG Comparison'!$B$2:$B$13,C$4)</f>
         <v>0.59199999999999997</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A7,'RAG Comparison'!$B$2:$B$13,D$4)</f>
         <v>0.66749999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="6">
+        <v>23</v>
+      </c>
+      <c r="B8" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A8,'RAG Comparison'!$B$2:$B$13,B$4)</f>
-        <v>0.76580000000000004</v>
-      </c>
-      <c r="C8" s="6">
+        <v>0.86199999999999999</v>
+      </c>
+      <c r="C8" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A8,'RAG Comparison'!$B$2:$B$13,C$4)</f>
         <v>0.71950000000000003</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <f>SUMIFS('RAG Comparison'!$C$2:$C$13,'RAG Comparison'!$A$2:$A$13,$A8,'RAG Comparison'!$B$2:$B$13,D$4)</f>
         <v>0.73319999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>25</v>
+      <c r="A12" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>16</v>
+      <c r="A13" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="B13" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A13,'RAG Comparison'!$B$2:$B$13,B$12)</f>
-        <v>0.84</v>
+        <v>1</v>
       </c>
       <c r="C13" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A13,'RAG Comparison'!$B$2:$B$13,C$12)</f>
@@ -10987,82 +9957,82 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="6">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A14,'RAG Comparison'!$B$2:$B$13,B$12)</f>
-        <v>0.87729999999999997</v>
-      </c>
-      <c r="C14" s="6">
+        <v>0.93030000000000002</v>
+      </c>
+      <c r="C14" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A14,'RAG Comparison'!$B$2:$B$13,C$12)</f>
         <v>0.72399999999999998</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A14,'RAG Comparison'!$B$2:$B$13,D$12)</f>
         <v>0.72</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="6">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A15,'RAG Comparison'!$B$2:$B$13,B$12)</f>
-        <v>0.94799999999999995</v>
-      </c>
-      <c r="C15" s="6">
+        <v>0.97199999999999998</v>
+      </c>
+      <c r="C15" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A15,'RAG Comparison'!$B$2:$B$13,C$12)</f>
         <v>0.82330000000000003</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A15,'RAG Comparison'!$B$2:$B$13,D$12)</f>
         <v>0.81530000000000002</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="6">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A16,'RAG Comparison'!$B$2:$B$13,B$12)</f>
-        <v>0.87</v>
-      </c>
-      <c r="C16" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="C16" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A16,'RAG Comparison'!$B$2:$B$13,C$12)</f>
         <v>0.96330000000000005</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="7">
         <f>SUMIFS('RAG Comparison'!$D$2:$D$13,'RAG Comparison'!$A$2:$A$13,$A16,'RAG Comparison'!$B$2:$B$13,D$12)</f>
         <v>0.94669999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>25</v>
+      <c r="A20" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="8" t="s">
-        <v>16</v>
+      <c r="A21" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="B21" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A21,'RAG Comparison'!$B$2:$B$13,B$20)</f>
-        <v>0.72</v>
+        <v>0.86</v>
       </c>
       <c r="C21" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A21,'RAG Comparison'!$B$2:$B$13,C$20)</f>
@@ -11074,169 +10044,169 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="6">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A22,'RAG Comparison'!$B$2:$B$13,B$20)</f>
-        <v>0.94</v>
-      </c>
-      <c r="C22" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="C22" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A22,'RAG Comparison'!$B$2:$B$13,C$20)</f>
         <v>0.85</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A22,'RAG Comparison'!$B$2:$B$13,D$20)</f>
         <v>0.84</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="6">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A23,'RAG Comparison'!$B$2:$B$13,B$20)</f>
-        <v>0.96</v>
-      </c>
-      <c r="C23" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="C23" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A23,'RAG Comparison'!$B$2:$B$13,C$20)</f>
         <v>0.81</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A23,'RAG Comparison'!$B$2:$B$13,D$20)</f>
         <v>0.82</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" s="6">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A24,'RAG Comparison'!$B$2:$B$13,B$20)</f>
-        <v>0.84</v>
-      </c>
-      <c r="C24" s="6">
+        <v>0.94</v>
+      </c>
+      <c r="C24" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A24,'RAG Comparison'!$B$2:$B$13,C$20)</f>
         <v>0.94</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="7">
         <f>SUMIFS('RAG Comparison'!$F$2:$F$13,'RAG Comparison'!$A$2:$A$13,$A24,'RAG Comparison'!$B$2:$B$13,D$20)</f>
         <v>0.9</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
-        <v>25</v>
+      <c r="A28" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B29" s="11">
+      <c r="A29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A29,'RAG Comparison'!$B$2:$B$13,B$28)</f>
-        <v>4.4400000000000004</v>
-      </c>
-      <c r="C29" s="11">
+        <v>5</v>
+      </c>
+      <c r="C29" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A29,'RAG Comparison'!$B$2:$B$13,C$28)</f>
         <v>4.6399999999999997</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A29,'RAG Comparison'!$B$2:$B$13,D$28)</f>
         <v>4.5599999999999996</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="10">
+      <c r="A30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A30,'RAG Comparison'!$B$2:$B$13,B$28)</f>
-        <v>4.92</v>
-      </c>
-      <c r="C30" s="10">
+        <v>4.88</v>
+      </c>
+      <c r="C30" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A30,'RAG Comparison'!$B$2:$B$13,C$28)</f>
         <v>5</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A30,'RAG Comparison'!$B$2:$B$13,D$28)</f>
         <v>4.68</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B31" s="10">
+      <c r="A31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A31,'RAG Comparison'!$B$2:$B$13,B$28)</f>
         <v>5</v>
       </c>
-      <c r="C31" s="10">
+      <c r="C31" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A31,'RAG Comparison'!$B$2:$B$13,C$28)</f>
         <v>4.5199999999999996</v>
       </c>
-      <c r="D31" s="10">
+      <c r="D31" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A31,'RAG Comparison'!$B$2:$B$13,D$28)</f>
         <v>4.5599999999999996</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B32" s="10">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A32,'RAG Comparison'!$B$2:$B$13,B$28)</f>
-        <v>4.8</v>
-      </c>
-      <c r="C32" s="10">
+        <v>5</v>
+      </c>
+      <c r="C32" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A32,'RAG Comparison'!$B$2:$B$13,C$28)</f>
         <v>4.92</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="8">
         <f>SUMIFS('RAG Comparison'!$E$2:$E$13,'RAG Comparison'!$A$2:$A$13,$A32,'RAG Comparison'!$B$2:$B$13,D$28)</f>
         <v>4.88</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>25</v>
+      <c r="A36" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="8" t="s">
-        <v>16</v>
+      <c r="A37" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="B37" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A37,'RAG Comparison'!$B$2:$B$13,B$36)</f>
-        <v>0.44</v>
+        <v>0.52959999999999996</v>
       </c>
       <c r="C37" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A37,'RAG Comparison'!$B$2:$B$13,C$36)</f>
@@ -11248,401 +10218,314 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="6">
+      <c r="A38" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A38,'RAG Comparison'!$B$2:$B$13,B$36)</f>
-        <v>0.55600000000000005</v>
-      </c>
-      <c r="C38" s="6">
+        <v>0.52959999999999996</v>
+      </c>
+      <c r="C38" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A38,'RAG Comparison'!$B$2:$B$13,C$36)</f>
         <v>0.41639999999999999</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A38,'RAG Comparison'!$B$2:$B$13,D$36)</f>
         <v>0.47320000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B39" s="6">
+      <c r="A39" t="s">
+        <v>22</v>
+      </c>
+      <c r="B39" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A39,'RAG Comparison'!$B$2:$B$13,B$36)</f>
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="C39" s="6">
+        <v>0.48880000000000001</v>
+      </c>
+      <c r="C39" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A39,'RAG Comparison'!$B$2:$B$13,C$36)</f>
         <v>0.45679999999999998</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A39,'RAG Comparison'!$B$2:$B$13,D$36)</f>
         <v>0.46279999999999999</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" s="6">
+      <c r="A40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A40,'RAG Comparison'!$B$2:$B$13,B$36)</f>
-        <v>0.58919999999999995</v>
-      </c>
-      <c r="C40" s="6">
+        <v>0.65959999999999996</v>
+      </c>
+      <c r="C40" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A40,'RAG Comparison'!$B$2:$B$13,C$36)</f>
         <v>0.68679999999999997</v>
       </c>
-      <c r="D40" s="6">
+      <c r="D40" s="7">
         <f>SUMIFS('RAG Comparison'!$G$2:$G$13,'RAG Comparison'!$A$2:$A$13,$A40,'RAG Comparison'!$B$2:$B$13,D$36)</f>
         <v>0.59079999999999999</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
-        <v>25</v>
+      <c r="A44" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B45" s="13">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,B$44)</f>
-        <v>7.9469999999999992E-3</v>
-      </c>
-      <c r="C45" s="13">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,C$44)</f>
+      <c r="A45" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B45" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,B$44)</f>
+        <v>8.9099999999999997E-4</v>
+      </c>
+      <c r="C45" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,C$44)</f>
         <v>7.4700000000000005E-4</v>
       </c>
-      <c r="D45" s="13">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,D$44)</f>
+      <c r="D45" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A45,'RAG Comparison'!$B$2:$B$13,D$44)</f>
         <v>6.9700000000000003E-4</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B46" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,B$44)</f>
-        <v>9.3489999999999997E-3</v>
-      </c>
-      <c r="C46" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,C$44)</f>
+      <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,B$44)</f>
+        <v>1.33E-3</v>
+      </c>
+      <c r="C46" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,C$44)</f>
         <v>8.8500000000000004E-4</v>
       </c>
-      <c r="D46" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,D$44)</f>
+      <c r="D46" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A46,'RAG Comparison'!$B$2:$B$13,D$44)</f>
         <v>8.9800000000000004E-4</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B47" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,B$44)</f>
-        <v>8.6020000000000003E-3</v>
-      </c>
-      <c r="C47" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,C$44)</f>
+      <c r="A47" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,B$44)</f>
+        <v>1.32E-3</v>
+      </c>
+      <c r="C47" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,C$44)</f>
         <v>8.2299999999999995E-4</v>
       </c>
-      <c r="D47" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,D$44)</f>
+      <c r="D47" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A47,'RAG Comparison'!$B$2:$B$13,D$44)</f>
         <v>8.7200000000000005E-4</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,B$44)</f>
-        <v>8.9840000000000007E-3</v>
-      </c>
-      <c r="C48" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,C$44)</f>
+      <c r="A48" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,B$44)</f>
+        <v>1.0510000000000001E-3</v>
+      </c>
+      <c r="C48" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,C$44)</f>
         <v>7.5600000000000005E-4</v>
       </c>
-      <c r="D48" s="12">
-        <f>SUMIFS('RAG Comparison'!$K$2:$K$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,D$44)</f>
+      <c r="D48" s="9">
+        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A48,'RAG Comparison'!$B$2:$B$13,D$44)</f>
         <v>7.9100000000000004E-4</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
-        <v>25</v>
+      <c r="A52" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" s="13">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,B$52)</f>
-        <v>5.2700000000000002E-4</v>
-      </c>
-      <c r="C53" s="13">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,C$52)</f>
+      <c r="A53" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,B$52)</f>
+        <v>8.9099999999999997E-4</v>
+      </c>
+      <c r="C53" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,C$52)</f>
         <v>7.4700000000000005E-4</v>
       </c>
-      <c r="D53" s="13">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,D$52)</f>
+      <c r="D53" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A53,'RAG Comparison'!$B$2:$B$13,D$52)</f>
         <v>6.9700000000000003E-4</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B54" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,B$52)</f>
-        <v>9.9400000000000009E-4</v>
-      </c>
-      <c r="C54" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,C$52)</f>
+      <c r="A54" t="s">
+        <v>21</v>
+      </c>
+      <c r="B54" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,B$52)</f>
+        <v>1.33E-3</v>
+      </c>
+      <c r="C54" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,C$52)</f>
         <v>8.8500000000000004E-4</v>
       </c>
-      <c r="D54" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,D$52)</f>
+      <c r="D54" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A54,'RAG Comparison'!$B$2:$B$13,D$52)</f>
         <v>8.9800000000000004E-4</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B55" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,B$52)</f>
-        <v>8.8599999999999996E-4</v>
-      </c>
-      <c r="C55" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,C$52)</f>
+      <c r="A55" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,B$52)</f>
+        <v>1.32E-3</v>
+      </c>
+      <c r="C55" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,C$52)</f>
         <v>8.2299999999999995E-4</v>
       </c>
-      <c r="D55" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,D$52)</f>
+      <c r="D55" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A55,'RAG Comparison'!$B$2:$B$13,D$52)</f>
         <v>8.7200000000000005E-4</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B56" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,B$52)</f>
-        <v>6.8400000000000004E-4</v>
-      </c>
-      <c r="C56" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,C$52)</f>
+      <c r="A56" t="s">
+        <v>23</v>
+      </c>
+      <c r="B56" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,B$52)</f>
+        <v>1.0510000000000001E-3</v>
+      </c>
+      <c r="C56" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,C$52)</f>
         <v>7.5600000000000005E-4</v>
       </c>
-      <c r="D56" s="12">
-        <f>SUMIFS('RAG Comparison'!$O$2:$O$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,D$52)</f>
+      <c r="D56" s="9">
+        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A56,'RAG Comparison'!$B$2:$B$13,D$52)</f>
         <v>7.9100000000000004E-4</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="4" t="s">
-        <v>25</v>
+      <c r="A60" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B61" s="15">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,B$60)</f>
-        <v>30420.48</v>
-      </c>
-      <c r="C61" s="15">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,C$60)</f>
+      <c r="A61" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B61" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,B$60)</f>
+        <v>41182.92</v>
+      </c>
+      <c r="C61" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,C$60)</f>
         <v>2243.88</v>
       </c>
-      <c r="D61" s="15">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,D$60)</f>
+      <c r="D61" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A61,'RAG Comparison'!$B$2:$B$13,D$60)</f>
         <v>2126.12</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B62" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,B$60)</f>
-        <v>35315.279999999999</v>
-      </c>
-      <c r="C62" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,C$60)</f>
+      <c r="A62" t="s">
+        <v>21</v>
+      </c>
+      <c r="B62" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,B$60)</f>
+        <v>40293.08</v>
+      </c>
+      <c r="C62" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,C$60)</f>
         <v>2297.3200000000002</v>
       </c>
-      <c r="D62" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,D$60)</f>
+      <c r="D62" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A62,'RAG Comparison'!$B$2:$B$13,D$60)</f>
         <v>2391.6799999999998</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B63" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,B$60)</f>
-        <v>32730.76</v>
-      </c>
-      <c r="C63" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,C$60)</f>
+      <c r="A63" t="s">
+        <v>22</v>
+      </c>
+      <c r="B63" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,B$60)</f>
+        <v>40745.599999999999</v>
+      </c>
+      <c r="C63" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,C$60)</f>
         <v>2285.2800000000002</v>
       </c>
-      <c r="D63" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,D$60)</f>
+      <c r="D63" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A63,'RAG Comparison'!$B$2:$B$13,D$60)</f>
         <v>2403.8000000000002</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B64" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,B$60)</f>
-        <v>34701.68</v>
-      </c>
-      <c r="C64" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,C$60)</f>
+      <c r="A64" t="s">
+        <v>23</v>
+      </c>
+      <c r="B64" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,B$60)</f>
+        <v>44095.88</v>
+      </c>
+      <c r="C64" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,C$60)</f>
         <v>2308.16</v>
       </c>
-      <c r="D64" s="14">
-        <f>SUMIFS('RAG Comparison'!$L$2:$L$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,D$60)</f>
-        <v>2378</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B69" s="15">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A69,'RAG Comparison'!$B$2:$B$13,B$68)</f>
-        <v>1374.52</v>
-      </c>
-      <c r="C69" s="15">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A69,'RAG Comparison'!$B$2:$B$13,C$68)</f>
-        <v>2243.88</v>
-      </c>
-      <c r="D69" s="15">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A69,'RAG Comparison'!$B$2:$B$13,D$68)</f>
-        <v>2126.12</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B70" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A70,'RAG Comparison'!$B$2:$B$13,B$68)</f>
-        <v>2514.6799999999998</v>
-      </c>
-      <c r="C70" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A70,'RAG Comparison'!$B$2:$B$13,C$68)</f>
-        <v>2297.3200000000002</v>
-      </c>
-      <c r="D70" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A70,'RAG Comparison'!$B$2:$B$13,D$68)</f>
-        <v>2391.6799999999998</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B71" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A71,'RAG Comparison'!$B$2:$B$13,B$68)</f>
-        <v>2076.88</v>
-      </c>
-      <c r="C71" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A71,'RAG Comparison'!$B$2:$B$13,C$68)</f>
-        <v>2285.2800000000002</v>
-      </c>
-      <c r="D71" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A71,'RAG Comparison'!$B$2:$B$13,D$68)</f>
-        <v>2403.8000000000002</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B72" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A72,'RAG Comparison'!$B$2:$B$13,B$68)</f>
-        <v>1875.72</v>
-      </c>
-      <c r="C72" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A72,'RAG Comparison'!$B$2:$B$13,C$68)</f>
-        <v>2308.16</v>
-      </c>
-      <c r="D72" s="14">
-        <f>SUMIFS('RAG Comparison'!$P$2:$P$13,'RAG Comparison'!$A$2:$A$13,$A72,'RAG Comparison'!$B$2:$B$13,D$68)</f>
+      <c r="D64" s="10">
+        <f>SUMIFS('RAG Comparison'!$M$2:$M$13,'RAG Comparison'!$A$2:$A$13,$A64,'RAG Comparison'!$B$2:$B$13,D$60)</f>
         <v>2378</v>
       </c>
     </row>

</xml_diff>